<commit_message>
Add ComposeWeekly feature with Gemini insights and Docker deployment setup
</commit_message>
<xml_diff>
--- a/specs.xlsx
+++ b/specs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cherifbenham/code/amadeus_ci_newsletter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B4A4DA2-712B-8F43-BF90-8D91B6EF6B17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3691A2B4-8CC0-7A40-83EC-CEBAE71D0697}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16940" activeTab="1" xr2:uid="{5E76CF1C-9E11-6E45-B6B5-E55FE503A1FD}"/>
+    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16940" xr2:uid="{5E76CF1C-9E11-6E45-B6B5-E55FE503A1FD}"/>
   </bookViews>
   <sheets>
     <sheet name="weekly selection" sheetId="1" r:id="rId1"/>
@@ -205,16 +205,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>225442</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>142782</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>263016</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>195385</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>670168</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>133088</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>602535</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>185691</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -237,7 +237,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5057454" y="2577575"/>
+          <a:off x="2742898" y="3441776"/>
           <a:ext cx="5359400" cy="2019300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -251,7 +251,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>

</xml_diff>